<commit_message>
Stop the first card on Needs attention doing nothing
Account changes are the one queue that lives on the Needs attention page
itself, but the card was built from the same list as all the others and
linked to /admin/approvals — the page the reader is already on. Clicking
it left the URL and the scroll position exactly where they were, so it
read as broken. The queue underneath was working the whole time, with the
request and its Approve button rendered correctly.

It jumps to the section below now, and the card says "below" so it no
longer promises to take you somewhere else.

Also checked the other two cards actually resolve to real screens rather
than assuming they did.

Verified: the card's href, the URL after clicking, and — at a window
short enough for the section to start off-screen — that it scrolls 208px
and brings the request card into view.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Things That Need Attention.xlsx
+++ b/docs/Things That Need Attention.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1528" uniqueCount="766">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1536" uniqueCount="770">
   <si>
     <t>AussieMed — things that need attention</t>
   </si>
@@ -1980,6 +1980,18 @@
   </si>
   <si>
     <t>Built 17 Aug 2026 at the client's request. The arithmetic moved into a pure cutoff.ts shared by both sides, so the countdown a buyer sees and the instant the buying run pools against cannot disagree — a customer told they had twenty minutes and then missing the run would be a promise broken by a rounding difference, and there is now a test asserting the two never diverge. Admin gets a picker in Settings showing the exact sentence a buyer will read, before saving rather than after, because this one number is a promise made to every customer. Buyers get a bar under the header on every storefront page, including the 404: the server renders the deadline, which is true whenever the page was built, and the countdown appears after mount and ticks, so there is no hydration mismatch and no stale number. Once the deadline passes the bar corrects its own wording rather than waiting for a refresh that may never come. Two defects the tests caught before shipping: parseCutoffHour returned 0 for an empty field, because Number('') is 0 and 0 is a valid hour — an empty form would have quietly moved every buyer's deadline to midnight; and the invariant test between the two directions found that they name the same instant when standing exactly on the cutoff, which is correct and now documented, with the display erring toward telling a buyer they have missed it rather than the reverse. Note: there is no weekend or holiday rule — the cutoff is daily. If the buying run does not happen at weekends, that is a business rule nobody has stated and it needs its own decision.</t>
+  </si>
+  <si>
+    <t>BE-50</t>
+  </si>
+  <si>
+    <t>The first card on Needs attention did nothing when clicked</t>
+  </si>
+  <si>
+    <t>Account changes are the one queue that lives on the Needs attention page itself, but its card was built from the same list as the others and linked to /admin/approvals — the page the reader was already on. Clicking it changed nothing and moved nothing, so it read as a broken feature. The queue underneath was working the whole time.</t>
+  </si>
+  <si>
+    <t>Reported by the client 17 Aug 2026 and reproduced immediately: the card's href was the current path, and clicking left both the URL and the scroll position untouched. It now jumps to the section below and says so on the card, so it no longer looks like a link that goes somewhere else. Confirmed the other cards resolve to real screens rather than being assumed to.</t>
   </si>
   <si>
     <t>DA-23</t>
@@ -2821,7 +2833,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="3">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -2845,7 +2857,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="3">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -5925,7 +5937,7 @@
   <sheetPr>
     <tabColor rgb="FF146C43"/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -7268,7 +7280,7 @@
         <v>655</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C52" s="6" t="s">
         <v>656</v>
@@ -7276,8 +7288,8 @@
       <c r="D52" s="6" t="s">
         <v>657</v>
       </c>
-      <c r="E52" s="7" t="s">
-        <v>13</v>
+      <c r="E52" s="6" t="s">
+        <v>16</v>
       </c>
       <c r="F52" s="9" t="s">
         <v>102</v>
@@ -7294,7 +7306,7 @@
         <v>659</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>332</v>
+        <v>19</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>660</v>
@@ -7302,8 +7314,8 @@
       <c r="D53" s="6" t="s">
         <v>661</v>
       </c>
-      <c r="E53" s="6" t="s">
-        <v>16</v>
+      <c r="E53" s="7" t="s">
+        <v>13</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>102</v>
@@ -7364,21 +7376,21 @@
         <v>332</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>449</v>
+        <v>670</v>
       </c>
     </row>
     <row r="56" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="7" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B56" s="6" t="s">
         <v>332</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>16</v>
@@ -7390,7 +7402,7 @@
         <v>332</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>673</v>
+        <v>449</v>
       </c>
     </row>
     <row r="57" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -7502,7 +7514,7 @@
         <v>690</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>21</v>
+        <v>332</v>
       </c>
       <c r="C61" s="6" t="s">
         <v>691</v>
@@ -7528,7 +7540,7 @@
         <v>694</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>695</v>
@@ -7606,7 +7618,7 @@
         <v>706</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C65" s="6" t="s">
         <v>707</v>
@@ -7736,7 +7748,7 @@
         <v>726</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C70" s="6" t="s">
         <v>727</v>
@@ -7762,7 +7774,7 @@
         <v>730</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C71" s="6" t="s">
         <v>731</v>
@@ -7773,8 +7785,8 @@
       <c r="E71" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F71" s="10" t="s">
-        <v>260</v>
+      <c r="F71" s="9" t="s">
+        <v>102</v>
       </c>
       <c r="G71" s="11" t="s">
         <v>332</v>
@@ -7866,7 +7878,7 @@
         <v>746</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C75" s="6" t="s">
         <v>747</v>
@@ -7874,8 +7886,8 @@
       <c r="D75" s="6" t="s">
         <v>748</v>
       </c>
-      <c r="E75" s="7" t="s">
-        <v>13</v>
+      <c r="E75" s="6" t="s">
+        <v>16</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>260</v>
@@ -7926,8 +7938,8 @@
       <c r="D77" s="6" t="s">
         <v>756</v>
       </c>
-      <c r="E77" s="6" t="s">
-        <v>16</v>
+      <c r="E77" s="7" t="s">
+        <v>13</v>
       </c>
       <c r="F77" s="10" t="s">
         <v>260</v>
@@ -7944,7 +7956,7 @@
         <v>758</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="C78" s="6" t="s">
         <v>759</v>
@@ -7970,7 +7982,7 @@
         <v>762</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C79" s="6" t="s">
         <v>763</v>
@@ -7991,8 +8003,34 @@
         <v>765</v>
       </c>
     </row>
+    <row r="80" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="7" t="s">
+        <v>766</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>767</v>
+      </c>
+      <c r="D80" s="6" t="s">
+        <v>768</v>
+      </c>
+      <c r="E80" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F80" s="10" t="s">
+        <v>260</v>
+      </c>
+      <c r="G80" s="11" t="s">
+        <v>332</v>
+      </c>
+      <c r="H80" s="6" t="s">
+        <v>769</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H79"/>
+  <autoFilter ref="A1:H80"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Record the two answers that needed no code
The cutoff stays daily (DEC-28) and email stays plain text (DEC-30),
both asked with their alternatives and both answered by the client on
18 Aug. Recorded as decisions rather than left as notes inside finished
rows, because a question that was asked and answered should not read
like a question nobody got to.

DEC-28 carries what daily commits the business to: the storefront
countdown tells a clinic on Saturday afternoon that ordering now makes
today's run, so somebody has to work the weekend drafts for that to be
true. Nothing reaches a supplier unattended, since auto-send is off.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Things That Need Attention.xlsx
+++ b/docs/Things That Need Attention.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1833" uniqueCount="919">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1841" uniqueCount="923">
   <si>
     <t>AussieMed — things that need attention</t>
   </si>
@@ -1310,6 +1310,18 @@
     <t>Done the same day. The customer's bulk .xlsx of invoices and the per-invoice spreadsheet link are gone, along with src/lib/invoice-workbook.ts, the download actions and the button component. invoicesForPeriod went with them: the bulk download was its only caller, and a query nobody calls is a query nobody maintains. WHAT CUSTOMERS STILL HAVE: the Spending tab itself, with the period in the URL so it can be bookmarked and shared, the breakdown by month, category, branch and person, and a printable page per invoice their browser saves as a PDF. WHAT THIS COSTS: an accountant reconciling a quarter now retypes figures rather than pivoting them, and there is still no way to take many invoices at once. That is the trade the client chose, and DF-05 already carries the wider question of downloadable documents. The exceljs dependency STAYS — the admin catalogue upload template (BE-04), the supplier's supply-terms workbook (BE-21) and the generated register spreadsheet all use it, and all three are inputs the business actually works from rather than exports nobody asked for.</t>
   </si>
   <si>
+    <t>DEC-30</t>
+  </si>
+  <si>
+    <t>Email stays plain text</t>
+  </si>
+  <si>
+    <t>Every message the platform sends is plain text. It was built that way because the alternative meant inventing a brand email look nobody had approved, and the question was left open rather than decided by default.</t>
+  </si>
+  <si>
+    <t>Decided by the client 18 Aug 2026, asked with the alternatives of a branded HTML layout and HTML for customer-facing mail only. Their answer: leave it plain. The reasons that make this a decision rather than a shortcut: plain text renders on every client, on a phone and through a hospital mail filter; it cannot carry a tracking pixel, which matters when the recipients are clinics; and it reads as though a person wrote it, which suits a trade supplier. What it gives up is a logo and any layout beyond line breaks, so an order confirmation is a list rather than a table. All the wording lives in src/lib/email-message.ts, which imports nothing at runtime and is tested on its own, so adding an HTML body later is a change in one file rather than a rewrite — the seam is already there if a designer ever supplies a template.</t>
+  </si>
+  <si>
     <t>DA-09</t>
   </si>
   <si>
@@ -1910,7 +1922,7 @@
     <t>OTP verification, order confirmation, restock alerts, supplier notifications to both primary and secondary addresses.</t>
   </si>
   <si>
-    <t>Built 16 Aug 2026. A seam like storage.ts, and for the same reason: no provider has been chosen and hosting is IN-01, so everything that could touch a network is confined to mailer.ts. The default driver writes readable .eml files to a gitignored outbox folder, which is right for a laptop and right for a demo — nothing escapes to a real inbox while the catalogue is still seeded test data — and adding Postmark, SES or SMTP means writing one more driver and setting MAIL_DRIVER, with no calling code changed. An smtp driver exists and throws loudly rather than accepting mail and quietly dropping it, which would recreate the exact bug this closes. The wording lives in email-message.ts, which is pure and imports nothing at runtime, so what a customer reads can be tested without a mail server and cannot change with a second driver. Platform conventions are enforced there rather than remembered at each call site: AED in English, VAT shown separately, reference number and never order number, and times written in Asia/Dubai because 23:30 UTC is the following day for the person reading it. Five kinds are wired. Order confirmation on checkout, sent after the transaction commits so a full mailbox cannot lose an order. Restock alerts on the moment a pack comes back in stock — the one automated client-facing message the design allows, fired only on the transition and stamped per subscription so nobody is told twice. Account change decisions to whoever raised them, approved or refused, carrying our reason. Purchase orders to the supplier, to both the primary and secondary addresses because that is what the second address is for, sent separately so one bad address cannot suppress the other. Staff alerts, which are internal and therefore not outreach. The two privacy rules are unit tested on the templates and checked again against what was actually stored: no supplier email names a customer, no customer email names a supplier. A purchase order carries quantities and codes and not a single price. Not built, and deliberately: OTP verification, which is part of a sign-in flow that does not exist yet, and HTML bodies, which are a client design decision. Plain text arrives in every client, cannot break in Outlook, and cannot carry a tracking pixel.</t>
+    <t>Built 16 Aug 2026. A seam like storage.ts, and for the same reason: no provider has been chosen and hosting is IN-01, so everything that could touch a network is confined to mailer.ts. The default driver writes readable .eml files to a gitignored outbox folder, which is right for a laptop and right for a demo — nothing escapes to a real inbox while the catalogue is still seeded test data — and adding Postmark, SES or SMTP means writing one more driver and setting MAIL_DRIVER, with no calling code changed. An smtp driver exists and throws loudly rather than accepting mail and quietly dropping it, which would recreate the exact bug this closes. The wording lives in email-message.ts, which is pure and imports nothing at runtime, so what a customer reads can be tested without a mail server and cannot change with a second driver. Platform conventions are enforced there rather than remembered at each call site: AED in English, VAT shown separately, reference number and never order number, and times written in Asia/Dubai because 23:30 UTC is the following day for the person reading it. Five kinds are wired. Order confirmation on checkout, sent after the transaction commits so a full mailbox cannot lose an order. Restock alerts on the moment a pack comes back in stock — the one automated client-facing message the design allows, fired only on the transition and stamped per subscription so nobody is told twice. Account change decisions to whoever raised them, approved or refused, carrying our reason. Purchase orders to the supplier, to both the primary and secondary addresses because that is what the second address is for, sent separately so one bad address cannot suppress the other. Staff alerts, which are internal and therefore not outreach. The two privacy rules are unit tested on the templates and checked again against what was actually stored: no supplier email names a customer, no customer email names a supplier. A purchase order carries quantities and codes and not a single price. Not built, and deliberately: OTP verification, which is part of a sign-in flow that does not exist yet, and HTML bodies, which are a client design decision. Plain text arrives in every client, cannot break in Outlook, and cannot carry a tracking pixel. Answered by the client 18 Aug 2026: plain text stays. See DEC-30.</t>
   </si>
   <si>
     <t>BE-06</t>
@@ -3280,7 +3292,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="3">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3288,7 +3300,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="3">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -3304,7 +3316,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="3">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -5356,7 +5368,7 @@
   <sheetPr>
     <tabColor rgb="FF29387D"/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -6148,8 +6160,34 @@
         <v>430</v>
       </c>
     </row>
+    <row r="31" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="7" t="s">
+        <v>431</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>432</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>433</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F31" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="G31" s="11" t="s">
+        <v>317</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>434</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H30"/>
+  <autoFilter ref="A1:H31"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -6200,16 +6238,16 @@
     </row>
     <row r="2" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>13</v>
@@ -6221,21 +6259,21 @@
         <v>7</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
     </row>
     <row r="3" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="E3" s="6" t="s">
         <v>16</v>
@@ -6247,21 +6285,21 @@
         <v>7</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
     </row>
     <row r="4" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>16</v>
@@ -6273,21 +6311,21 @@
         <v>7</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>16</v>
@@ -6299,21 +6337,21 @@
         <v>7</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
     </row>
     <row r="6" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>16</v>
@@ -6330,16 +6368,16 @@
     </row>
     <row r="7" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>13</v>
@@ -6351,7 +6389,7 @@
         <v>7</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
     </row>
   </sheetData>
@@ -6406,16 +6444,16 @@
     </row>
     <row r="2" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>16</v>
@@ -6427,21 +6465,21 @@
         <v>317</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
     </row>
     <row r="3" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="E3" s="6" t="s">
         <v>16</v>
@@ -6453,21 +6491,21 @@
         <v>317</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
     </row>
     <row r="4" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>464</v>
+        <v>468</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>16</v>
@@ -6479,21 +6517,21 @@
         <v>317</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>16</v>
@@ -6505,21 +6543,21 @@
         <v>317</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
     </row>
     <row r="6" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>16</v>
@@ -6531,21 +6569,21 @@
         <v>317</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>16</v>
@@ -6557,21 +6595,21 @@
         <v>317</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>16</v>
@@ -6583,21 +6621,21 @@
         <v>317</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
     </row>
     <row r="9" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>16</v>
@@ -6609,21 +6647,21 @@
         <v>317</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
     </row>
     <row r="10" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>16</v>
@@ -6635,21 +6673,21 @@
         <v>317</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
     </row>
     <row r="11" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>16</v>
@@ -6661,21 +6699,21 @@
         <v>317</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>493</v>
+        <v>497</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>16</v>
@@ -6687,21 +6725,21 @@
         <v>317</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
     </row>
     <row r="13" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>16</v>
@@ -6713,21 +6751,21 @@
         <v>317</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
     </row>
     <row r="14" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>16</v>
@@ -6739,21 +6777,21 @@
         <v>317</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
     </row>
     <row r="15" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>16</v>
@@ -6765,21 +6803,21 @@
         <v>317</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
     </row>
     <row r="16" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>16</v>
@@ -6791,21 +6829,21 @@
         <v>317</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>513</v>
+        <v>517</v>
       </c>
     </row>
     <row r="17" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>516</v>
+        <v>520</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>16</v>
@@ -6817,21 +6855,21 @@
         <v>317</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
     </row>
     <row r="18" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
-        <v>518</v>
+        <v>522</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>16</v>
@@ -6843,21 +6881,21 @@
         <v>317</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>521</v>
+        <v>525</v>
       </c>
     </row>
     <row r="19" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>523</v>
+        <v>527</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>524</v>
+        <v>528</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>16</v>
@@ -6869,21 +6907,21 @@
         <v>317</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>525</v>
+        <v>529</v>
       </c>
     </row>
     <row r="20" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
-        <v>526</v>
+        <v>530</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>16</v>
@@ -6895,21 +6933,21 @@
         <v>317</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
     </row>
     <row r="21" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>16</v>
@@ -6921,21 +6959,21 @@
         <v>317</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
     </row>
     <row r="22" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>16</v>
@@ -6947,21 +6985,21 @@
         <v>317</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
     </row>
     <row r="23" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>539</v>
+        <v>543</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>16</v>
@@ -6973,21 +7011,21 @@
         <v>317</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
     </row>
     <row r="24" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
-        <v>541</v>
+        <v>545</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>542</v>
+        <v>546</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>16</v>
@@ -6999,21 +7037,21 @@
         <v>317</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
     </row>
     <row r="25" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>545</v>
+        <v>549</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>16</v>
@@ -7025,21 +7063,21 @@
         <v>317</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>547</v>
+        <v>551</v>
       </c>
     </row>
     <row r="26" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
-        <v>548</v>
+        <v>552</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>550</v>
+        <v>554</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>16</v>
@@ -7051,21 +7089,21 @@
         <v>317</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
     </row>
     <row r="27" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>16</v>
@@ -7077,21 +7115,21 @@
         <v>317</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
     </row>
     <row r="28" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>558</v>
+        <v>562</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>16</v>
@@ -7103,21 +7141,21 @@
         <v>317</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
     </row>
     <row r="29" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>560</v>
+        <v>564</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>561</v>
+        <v>565</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="E29" s="6" t="s">
         <v>16</v>
@@ -7129,21 +7167,21 @@
         <v>317</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
     </row>
     <row r="30" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>566</v>
+        <v>570</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>16</v>
@@ -7155,21 +7193,21 @@
         <v>317</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
     </row>
     <row r="31" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>569</v>
+        <v>573</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>570</v>
+        <v>574</v>
       </c>
       <c r="E31" s="6" t="s">
         <v>16</v>
@@ -7181,21 +7219,21 @@
         <v>317</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
     </row>
     <row r="32" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
-        <v>572</v>
+        <v>576</v>
       </c>
       <c r="B32" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>16</v>
@@ -7207,21 +7245,21 @@
         <v>317</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
     </row>
     <row r="33" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="B33" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="E33" s="6" t="s">
         <v>16</v>
@@ -7233,21 +7271,21 @@
         <v>317</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
     </row>
     <row r="34" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
       <c r="B34" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>16</v>
@@ -7259,21 +7297,21 @@
         <v>317</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
     </row>
     <row r="35" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="B35" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>586</v>
+        <v>590</v>
       </c>
       <c r="E35" s="6" t="s">
         <v>16</v>
@@ -7285,21 +7323,21 @@
         <v>317</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>587</v>
+        <v>591</v>
       </c>
     </row>
     <row r="36" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="7" t="s">
-        <v>588</v>
+        <v>592</v>
       </c>
       <c r="B36" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>16</v>
@@ -7311,21 +7349,21 @@
         <v>317</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
     </row>
     <row r="37" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
-        <v>592</v>
+        <v>596</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>593</v>
+        <v>597</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
       <c r="E37" s="6" t="s">
         <v>16</v>
@@ -7337,21 +7375,21 @@
         <v>317</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>595</v>
+        <v>599</v>
       </c>
     </row>
     <row r="38" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="7" t="s">
-        <v>596</v>
+        <v>600</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>16</v>
@@ -7363,21 +7401,21 @@
         <v>317</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
     </row>
     <row r="39" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
       <c r="B39" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="E39" s="6" t="s">
         <v>16</v>
@@ -7389,21 +7427,21 @@
         <v>317</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
     </row>
     <row r="40" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="7" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="B40" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>16</v>
@@ -7415,21 +7453,21 @@
         <v>317</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
     </row>
     <row r="41" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
       <c r="B41" s="6" t="s">
         <v>23</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="E41" s="7" t="s">
         <v>13</v>
@@ -7441,21 +7479,21 @@
         <v>317</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
     </row>
     <row r="42" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="7" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
       <c r="B42" s="6" t="s">
         <v>20</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
       <c r="E42" s="7" t="s">
         <v>13</v>
@@ -7467,21 +7505,21 @@
         <v>317</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
     </row>
     <row r="43" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
       <c r="B43" s="6" t="s">
         <v>24</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>16</v>
@@ -7493,21 +7531,21 @@
         <v>317</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
     </row>
     <row r="44" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="7" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="B44" s="6" t="s">
         <v>18</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>16</v>
@@ -7519,21 +7557,21 @@
         <v>317</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
     </row>
     <row r="45" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="B45" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>625</v>
+        <v>629</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>16</v>
@@ -7545,21 +7583,21 @@
         <v>317</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
     </row>
     <row r="46" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="7" t="s">
-        <v>628</v>
+        <v>632</v>
       </c>
       <c r="B46" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>16</v>
@@ -7571,21 +7609,21 @@
         <v>317</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
     </row>
     <row r="47" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
       <c r="B47" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>16</v>
@@ -7597,21 +7635,21 @@
         <v>317</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
     </row>
     <row r="48" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
-        <v>636</v>
+        <v>640</v>
       </c>
       <c r="B48" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>637</v>
+        <v>641</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>16</v>
@@ -7623,21 +7661,21 @@
         <v>317</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
     </row>
     <row r="49" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
       <c r="B49" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>641</v>
+        <v>645</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>642</v>
+        <v>646</v>
       </c>
       <c r="E49" s="6" t="s">
         <v>16</v>
@@ -7649,21 +7687,21 @@
         <v>317</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
     </row>
     <row r="50" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
-        <v>644</v>
+        <v>648</v>
       </c>
       <c r="B50" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>646</v>
+        <v>650</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>16</v>
@@ -7675,21 +7713,21 @@
         <v>317</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>647</v>
+        <v>651</v>
       </c>
     </row>
     <row r="51" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="B51" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>16</v>
@@ -7701,21 +7739,21 @@
         <v>317</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
     </row>
     <row r="52" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="7" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="B52" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>16</v>
@@ -7727,21 +7765,21 @@
         <v>317</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
     </row>
     <row r="53" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
-        <v>656</v>
+        <v>660</v>
       </c>
       <c r="B53" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>657</v>
+        <v>661</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>658</v>
+        <v>662</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>16</v>
@@ -7753,21 +7791,21 @@
         <v>317</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
     </row>
     <row r="54" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="7" t="s">
-        <v>660</v>
+        <v>664</v>
       </c>
       <c r="B54" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>662</v>
+        <v>666</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>16</v>
@@ -7779,21 +7817,21 @@
         <v>317</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>663</v>
+        <v>667</v>
       </c>
     </row>
     <row r="55" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="B55" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="E55" s="6" t="s">
         <v>16</v>
@@ -7805,21 +7843,21 @@
         <v>317</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>667</v>
+        <v>671</v>
       </c>
     </row>
     <row r="56" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="7" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
       <c r="B56" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>670</v>
+        <v>674</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>16</v>
@@ -7831,21 +7869,21 @@
         <v>317</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
     </row>
     <row r="57" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="B57" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
       <c r="E57" s="6" t="s">
         <v>16</v>
@@ -7857,21 +7895,21 @@
         <v>317</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>675</v>
+        <v>679</v>
       </c>
     </row>
     <row r="58" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="7" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
       <c r="B58" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>677</v>
+        <v>681</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>678</v>
+        <v>682</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>16</v>
@@ -7883,21 +7921,21 @@
         <v>317</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>679</v>
+        <v>683</v>
       </c>
     </row>
     <row r="59" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
-        <v>680</v>
+        <v>684</v>
       </c>
       <c r="B59" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
       <c r="E59" s="6" t="s">
         <v>16</v>
@@ -7909,21 +7947,21 @@
         <v>317</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
     </row>
     <row r="60" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="7" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="B60" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>16</v>
@@ -7935,21 +7973,21 @@
         <v>317</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
     </row>
     <row r="61" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="B61" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>16</v>
@@ -7961,21 +7999,21 @@
         <v>317</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
     </row>
     <row r="62" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
       <c r="B62" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>694</v>
+        <v>698</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>16</v>
@@ -7987,21 +8025,21 @@
         <v>317</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>695</v>
+        <v>699</v>
       </c>
     </row>
     <row r="63" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
       <c r="B63" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>697</v>
+        <v>701</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>698</v>
+        <v>702</v>
       </c>
       <c r="E63" s="6" t="s">
         <v>16</v>
@@ -8013,21 +8051,21 @@
         <v>317</v>
       </c>
       <c r="H63" s="6" t="s">
-        <v>699</v>
+        <v>703</v>
       </c>
     </row>
     <row r="64" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
-        <v>700</v>
+        <v>704</v>
       </c>
       <c r="B64" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>701</v>
+        <v>705</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>702</v>
+        <v>706</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>16</v>
@@ -8039,21 +8077,21 @@
         <v>317</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>703</v>
+        <v>707</v>
       </c>
     </row>
     <row r="65" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
       <c r="B65" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>705</v>
+        <v>709</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>706</v>
+        <v>710</v>
       </c>
       <c r="E65" s="6" t="s">
         <v>16</v>
@@ -8065,21 +8103,21 @@
         <v>317</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>707</v>
+        <v>711</v>
       </c>
     </row>
     <row r="66" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="7" t="s">
-        <v>708</v>
+        <v>712</v>
       </c>
       <c r="B66" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>710</v>
+        <v>714</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>16</v>
@@ -8091,21 +8129,21 @@
         <v>317</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
     </row>
     <row r="67" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
-        <v>712</v>
+        <v>716</v>
       </c>
       <c r="B67" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>713</v>
+        <v>717</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="E67" s="7" t="s">
         <v>13</v>
@@ -8117,21 +8155,21 @@
         <v>317</v>
       </c>
       <c r="H67" s="6" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
     </row>
     <row r="68" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="B68" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>717</v>
+        <v>721</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>718</v>
+        <v>722</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>16</v>
@@ -8143,21 +8181,21 @@
         <v>317</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>719</v>
+        <v>723</v>
       </c>
     </row>
     <row r="69" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="B69" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>721</v>
+        <v>725</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>722</v>
+        <v>726</v>
       </c>
       <c r="E69" s="6" t="s">
         <v>16</v>
@@ -8169,21 +8207,21 @@
         <v>317</v>
       </c>
       <c r="H69" s="6" t="s">
-        <v>723</v>
+        <v>727</v>
       </c>
     </row>
     <row r="70" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
-        <v>724</v>
+        <v>728</v>
       </c>
       <c r="B70" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>725</v>
+        <v>729</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>16</v>
@@ -8195,21 +8233,21 @@
         <v>317</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
     </row>
     <row r="71" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
-        <v>728</v>
+        <v>732</v>
       </c>
       <c r="B71" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>729</v>
+        <v>733</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>730</v>
+        <v>734</v>
       </c>
       <c r="E71" s="6" t="s">
         <v>16</v>
@@ -8221,21 +8259,21 @@
         <v>317</v>
       </c>
       <c r="H71" s="6" t="s">
-        <v>731</v>
+        <v>735</v>
       </c>
     </row>
     <row r="72" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="7" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="B72" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>734</v>
+        <v>738</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>16</v>
@@ -8247,21 +8285,21 @@
         <v>317</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>735</v>
+        <v>739</v>
       </c>
     </row>
     <row r="73" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
-        <v>736</v>
+        <v>740</v>
       </c>
       <c r="B73" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>737</v>
+        <v>741</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>738</v>
+        <v>742</v>
       </c>
       <c r="E73" s="6" t="s">
         <v>16</v>
@@ -8273,21 +8311,21 @@
         <v>317</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>739</v>
+        <v>743</v>
       </c>
     </row>
     <row r="74" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="7" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="B74" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>742</v>
+        <v>746</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>16</v>
@@ -8299,21 +8337,21 @@
         <v>317</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
     </row>
     <row r="75" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="B75" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
       <c r="E75" s="6" t="s">
         <v>16</v>
@@ -8325,21 +8363,21 @@
         <v>317</v>
       </c>
       <c r="H75" s="6" t="s">
-        <v>746</v>
+        <v>750</v>
       </c>
     </row>
     <row r="76" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="7" t="s">
-        <v>747</v>
+        <v>751</v>
       </c>
       <c r="B76" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>748</v>
+        <v>752</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>16</v>
@@ -8351,21 +8389,21 @@
         <v>317</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>750</v>
+        <v>754</v>
       </c>
     </row>
     <row r="77" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
-        <v>751</v>
+        <v>755</v>
       </c>
       <c r="B77" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>752</v>
+        <v>756</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
       <c r="E77" s="6" t="s">
         <v>16</v>
@@ -8377,21 +8415,21 @@
         <v>317</v>
       </c>
       <c r="H77" s="6" t="s">
-        <v>754</v>
+        <v>758</v>
       </c>
     </row>
     <row r="78" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="7" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="B78" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>756</v>
+        <v>760</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>16</v>
@@ -8403,21 +8441,21 @@
         <v>317</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>758</v>
+        <v>762</v>
       </c>
     </row>
     <row r="79" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
-        <v>759</v>
+        <v>763</v>
       </c>
       <c r="B79" s="6" t="s">
         <v>317</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>760</v>
+        <v>764</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>761</v>
+        <v>765</v>
       </c>
       <c r="E79" s="6" t="s">
         <v>16</v>
@@ -8429,21 +8467,21 @@
         <v>317</v>
       </c>
       <c r="H79" s="6" t="s">
-        <v>762</v>
+        <v>766</v>
       </c>
     </row>
     <row r="80" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="7" t="s">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="B80" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>764</v>
+        <v>768</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>16</v>
@@ -8455,21 +8493,21 @@
         <v>317</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>766</v>
+        <v>770</v>
       </c>
     </row>
     <row r="81" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
-        <v>767</v>
+        <v>771</v>
       </c>
       <c r="B81" s="6" t="s">
         <v>26</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>768</v>
+        <v>772</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>769</v>
+        <v>773</v>
       </c>
       <c r="E81" s="6" t="s">
         <v>16</v>
@@ -8481,21 +8519,21 @@
         <v>317</v>
       </c>
       <c r="H81" s="6" t="s">
-        <v>770</v>
+        <v>774</v>
       </c>
     </row>
     <row r="82" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="7" t="s">
-        <v>771</v>
+        <v>775</v>
       </c>
       <c r="B82" s="6" t="s">
         <v>26</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>772</v>
+        <v>776</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>773</v>
+        <v>777</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>16</v>
@@ -8507,21 +8545,21 @@
         <v>317</v>
       </c>
       <c r="H82" s="6" t="s">
-        <v>774</v>
+        <v>778</v>
       </c>
     </row>
     <row r="83" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="7" t="s">
-        <v>775</v>
+        <v>779</v>
       </c>
       <c r="B83" s="6" t="s">
         <v>26</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>776</v>
+        <v>780</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>777</v>
+        <v>781</v>
       </c>
       <c r="E83" s="6" t="s">
         <v>16</v>
@@ -8533,21 +8571,21 @@
         <v>317</v>
       </c>
       <c r="H83" s="6" t="s">
-        <v>778</v>
+        <v>782</v>
       </c>
     </row>
     <row r="84" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="7" t="s">
-        <v>779</v>
+        <v>783</v>
       </c>
       <c r="B84" s="6" t="s">
         <v>28</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>780</v>
+        <v>784</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>781</v>
+        <v>785</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>16</v>
@@ -8559,21 +8597,21 @@
         <v>317</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>782</v>
+        <v>786</v>
       </c>
     </row>
     <row r="85" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="7" t="s">
-        <v>783</v>
+        <v>787</v>
       </c>
       <c r="B85" s="6" t="s">
         <v>28</v>
       </c>
       <c r="C85" s="6" t="s">
-        <v>784</v>
+        <v>788</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>785</v>
+        <v>789</v>
       </c>
       <c r="E85" s="6" t="s">
         <v>16</v>
@@ -8585,21 +8623,21 @@
         <v>317</v>
       </c>
       <c r="H85" s="6" t="s">
-        <v>786</v>
+        <v>790</v>
       </c>
     </row>
     <row r="86" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="7" t="s">
-        <v>787</v>
+        <v>791</v>
       </c>
       <c r="B86" s="6" t="s">
         <v>28</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>788</v>
+        <v>792</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>16</v>
@@ -8611,21 +8649,21 @@
         <v>317</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
     </row>
     <row r="87" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="7" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="B87" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>792</v>
+        <v>796</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>793</v>
+        <v>797</v>
       </c>
       <c r="E87" s="6" t="s">
         <v>16</v>
@@ -8637,21 +8675,21 @@
         <v>317</v>
       </c>
       <c r="H87" s="6" t="s">
-        <v>794</v>
+        <v>798</v>
       </c>
     </row>
     <row r="88" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="7" t="s">
-        <v>795</v>
+        <v>799</v>
       </c>
       <c r="B88" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C88" s="6" t="s">
-        <v>796</v>
+        <v>800</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>797</v>
+        <v>801</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>16</v>
@@ -8663,21 +8701,21 @@
         <v>317</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>798</v>
+        <v>802</v>
       </c>
     </row>
     <row r="89" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="7" t="s">
-        <v>799</v>
+        <v>803</v>
       </c>
       <c r="B89" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C89" s="6" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="D89" s="6" t="s">
-        <v>801</v>
+        <v>805</v>
       </c>
       <c r="E89" s="6" t="s">
         <v>16</v>
@@ -8689,21 +8727,21 @@
         <v>317</v>
       </c>
       <c r="H89" s="6" t="s">
-        <v>802</v>
+        <v>806</v>
       </c>
     </row>
     <row r="90" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="7" t="s">
-        <v>803</v>
+        <v>807</v>
       </c>
       <c r="B90" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C90" s="6" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>805</v>
+        <v>809</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>16</v>
@@ -8715,21 +8753,21 @@
         <v>317</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>806</v>
+        <v>810</v>
       </c>
     </row>
     <row r="91" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="7" t="s">
-        <v>807</v>
+        <v>811</v>
       </c>
       <c r="B91" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C91" s="6" t="s">
-        <v>808</v>
+        <v>812</v>
       </c>
       <c r="D91" s="6" t="s">
-        <v>809</v>
+        <v>813</v>
       </c>
       <c r="E91" s="6" t="s">
         <v>16</v>
@@ -8741,21 +8779,21 @@
         <v>317</v>
       </c>
       <c r="H91" s="6" t="s">
-        <v>810</v>
+        <v>814</v>
       </c>
     </row>
     <row r="92" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="7" t="s">
-        <v>811</v>
+        <v>815</v>
       </c>
       <c r="B92" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C92" s="6" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="D92" s="6" t="s">
-        <v>813</v>
+        <v>817</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>16</v>
@@ -8767,21 +8805,21 @@
         <v>317</v>
       </c>
       <c r="H92" s="6" t="s">
-        <v>814</v>
+        <v>818</v>
       </c>
     </row>
     <row r="93" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="7" t="s">
-        <v>815</v>
+        <v>819</v>
       </c>
       <c r="B93" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C93" s="6" t="s">
-        <v>816</v>
+        <v>820</v>
       </c>
       <c r="D93" s="6" t="s">
-        <v>817</v>
+        <v>821</v>
       </c>
       <c r="E93" s="6" t="s">
         <v>16</v>
@@ -8793,21 +8831,21 @@
         <v>317</v>
       </c>
       <c r="H93" s="6" t="s">
-        <v>818</v>
+        <v>822</v>
       </c>
     </row>
     <row r="94" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="7" t="s">
-        <v>819</v>
+        <v>823</v>
       </c>
       <c r="B94" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C94" s="6" t="s">
-        <v>820</v>
+        <v>824</v>
       </c>
       <c r="D94" s="6" t="s">
-        <v>821</v>
+        <v>825</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>16</v>
@@ -8819,21 +8857,21 @@
         <v>317</v>
       </c>
       <c r="H94" s="6" t="s">
-        <v>822</v>
+        <v>826</v>
       </c>
     </row>
     <row r="95" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="7" t="s">
-        <v>823</v>
+        <v>827</v>
       </c>
       <c r="B95" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C95" s="6" t="s">
-        <v>824</v>
+        <v>828</v>
       </c>
       <c r="D95" s="6" t="s">
-        <v>825</v>
+        <v>829</v>
       </c>
       <c r="E95" s="6" t="s">
         <v>16</v>
@@ -8845,21 +8883,21 @@
         <v>317</v>
       </c>
       <c r="H95" s="6" t="s">
-        <v>826</v>
+        <v>830</v>
       </c>
     </row>
     <row r="96" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="7" t="s">
-        <v>827</v>
+        <v>831</v>
       </c>
       <c r="B96" s="6" t="s">
         <v>24</v>
       </c>
       <c r="C96" s="6" t="s">
-        <v>828</v>
+        <v>832</v>
       </c>
       <c r="D96" s="6" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>16</v>
@@ -8871,21 +8909,21 @@
         <v>317</v>
       </c>
       <c r="H96" s="6" t="s">
-        <v>830</v>
+        <v>834</v>
       </c>
     </row>
     <row r="97" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="7" t="s">
-        <v>831</v>
+        <v>835</v>
       </c>
       <c r="B97" s="6" t="s">
         <v>24</v>
       </c>
       <c r="C97" s="6" t="s">
-        <v>832</v>
+        <v>836</v>
       </c>
       <c r="D97" s="6" t="s">
-        <v>833</v>
+        <v>837</v>
       </c>
       <c r="E97" s="6" t="s">
         <v>16</v>
@@ -8897,21 +8935,21 @@
         <v>317</v>
       </c>
       <c r="H97" s="6" t="s">
-        <v>834</v>
+        <v>838</v>
       </c>
     </row>
     <row r="98" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="7" t="s">
-        <v>835</v>
+        <v>839</v>
       </c>
       <c r="B98" s="6" t="s">
         <v>24</v>
       </c>
       <c r="C98" s="6" t="s">
-        <v>836</v>
+        <v>840</v>
       </c>
       <c r="D98" s="6" t="s">
-        <v>837</v>
+        <v>841</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>16</v>
@@ -8923,21 +8961,21 @@
         <v>317</v>
       </c>
       <c r="H98" s="6" t="s">
-        <v>838</v>
+        <v>842</v>
       </c>
     </row>
     <row r="99" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="7" t="s">
-        <v>839</v>
+        <v>843</v>
       </c>
       <c r="B99" s="6" t="s">
         <v>24</v>
       </c>
       <c r="C99" s="6" t="s">
-        <v>840</v>
+        <v>844</v>
       </c>
       <c r="D99" s="6" t="s">
-        <v>841</v>
+        <v>845</v>
       </c>
       <c r="E99" s="6" t="s">
         <v>16</v>
@@ -8949,21 +8987,21 @@
         <v>317</v>
       </c>
       <c r="H99" s="6" t="s">
-        <v>842</v>
+        <v>846</v>
       </c>
     </row>
     <row r="100" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="7" t="s">
-        <v>843</v>
+        <v>847</v>
       </c>
       <c r="B100" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C100" s="6" t="s">
-        <v>844</v>
+        <v>848</v>
       </c>
       <c r="D100" s="6" t="s">
-        <v>845</v>
+        <v>849</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>16</v>
@@ -8975,21 +9013,21 @@
         <v>317</v>
       </c>
       <c r="H100" s="6" t="s">
-        <v>846</v>
+        <v>850</v>
       </c>
     </row>
     <row r="101" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="7" t="s">
-        <v>847</v>
+        <v>851</v>
       </c>
       <c r="B101" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C101" s="6" t="s">
-        <v>848</v>
+        <v>852</v>
       </c>
       <c r="D101" s="6" t="s">
-        <v>849</v>
+        <v>853</v>
       </c>
       <c r="E101" s="6" t="s">
         <v>16</v>
@@ -9001,21 +9039,21 @@
         <v>317</v>
       </c>
       <c r="H101" s="6" t="s">
-        <v>850</v>
+        <v>854</v>
       </c>
     </row>
     <row r="102" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="7" t="s">
-        <v>851</v>
+        <v>855</v>
       </c>
       <c r="B102" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C102" s="6" t="s">
-        <v>852</v>
+        <v>856</v>
       </c>
       <c r="D102" s="6" t="s">
-        <v>853</v>
+        <v>857</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>16</v>
@@ -9027,21 +9065,21 @@
         <v>317</v>
       </c>
       <c r="H102" s="6" t="s">
-        <v>854</v>
+        <v>858</v>
       </c>
     </row>
     <row r="103" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="7" t="s">
-        <v>855</v>
+        <v>859</v>
       </c>
       <c r="B103" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C103" s="6" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="D103" s="6" t="s">
-        <v>857</v>
+        <v>861</v>
       </c>
       <c r="E103" s="6" t="s">
         <v>16</v>
@@ -9053,21 +9091,21 @@
         <v>317</v>
       </c>
       <c r="H103" s="6" t="s">
-        <v>858</v>
+        <v>862</v>
       </c>
     </row>
     <row r="104" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="7" t="s">
-        <v>859</v>
+        <v>863</v>
       </c>
       <c r="B104" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C104" s="6" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="D104" s="6" t="s">
-        <v>861</v>
+        <v>865</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>16</v>
@@ -9079,21 +9117,21 @@
         <v>317</v>
       </c>
       <c r="H104" s="6" t="s">
-        <v>862</v>
+        <v>866</v>
       </c>
     </row>
     <row r="105" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="7" t="s">
-        <v>863</v>
+        <v>867</v>
       </c>
       <c r="B105" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C105" s="6" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="D105" s="6" t="s">
-        <v>865</v>
+        <v>869</v>
       </c>
       <c r="E105" s="6" t="s">
         <v>16</v>
@@ -9105,21 +9143,21 @@
         <v>317</v>
       </c>
       <c r="H105" s="6" t="s">
-        <v>866</v>
+        <v>870</v>
       </c>
     </row>
     <row r="106" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="7" t="s">
-        <v>867</v>
+        <v>871</v>
       </c>
       <c r="B106" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C106" s="6" t="s">
-        <v>868</v>
+        <v>872</v>
       </c>
       <c r="D106" s="6" t="s">
-        <v>869</v>
+        <v>873</v>
       </c>
       <c r="E106" s="7" t="s">
         <v>13</v>
@@ -9131,21 +9169,21 @@
         <v>317</v>
       </c>
       <c r="H106" s="6" t="s">
-        <v>870</v>
+        <v>874</v>
       </c>
     </row>
     <row r="107" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="7" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="B107" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C107" s="6" t="s">
-        <v>872</v>
+        <v>876</v>
       </c>
       <c r="D107" s="6" t="s">
-        <v>873</v>
+        <v>877</v>
       </c>
       <c r="E107" s="7" t="s">
         <v>13</v>
@@ -9157,21 +9195,21 @@
         <v>317</v>
       </c>
       <c r="H107" s="6" t="s">
-        <v>874</v>
+        <v>878</v>
       </c>
     </row>
     <row r="108" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="7" t="s">
-        <v>875</v>
+        <v>879</v>
       </c>
       <c r="B108" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C108" s="6" t="s">
-        <v>876</v>
+        <v>880</v>
       </c>
       <c r="D108" s="6" t="s">
-        <v>877</v>
+        <v>881</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>16</v>
@@ -9183,21 +9221,21 @@
         <v>317</v>
       </c>
       <c r="H108" s="6" t="s">
-        <v>878</v>
+        <v>882</v>
       </c>
     </row>
     <row r="109" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="7" t="s">
-        <v>879</v>
+        <v>883</v>
       </c>
       <c r="B109" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C109" s="6" t="s">
-        <v>880</v>
+        <v>884</v>
       </c>
       <c r="D109" s="6" t="s">
-        <v>881</v>
+        <v>885</v>
       </c>
       <c r="E109" s="6" t="s">
         <v>16</v>
@@ -9209,21 +9247,21 @@
         <v>317</v>
       </c>
       <c r="H109" s="6" t="s">
-        <v>882</v>
+        <v>886</v>
       </c>
     </row>
     <row r="110" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="7" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="B110" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C110" s="6" t="s">
-        <v>884</v>
+        <v>888</v>
       </c>
       <c r="D110" s="6" t="s">
-        <v>885</v>
+        <v>889</v>
       </c>
       <c r="E110" s="6" t="s">
         <v>16</v>
@@ -9235,21 +9273,21 @@
         <v>317</v>
       </c>
       <c r="H110" s="6" t="s">
-        <v>886</v>
+        <v>890</v>
       </c>
     </row>
     <row r="111" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="7" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="B111" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C111" s="6" t="s">
-        <v>888</v>
+        <v>892</v>
       </c>
       <c r="D111" s="6" t="s">
-        <v>889</v>
+        <v>893</v>
       </c>
       <c r="E111" s="6" t="s">
         <v>16</v>
@@ -9261,21 +9299,21 @@
         <v>317</v>
       </c>
       <c r="H111" s="6" t="s">
-        <v>890</v>
+        <v>894</v>
       </c>
     </row>
     <row r="112" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="7" t="s">
-        <v>891</v>
+        <v>895</v>
       </c>
       <c r="B112" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C112" s="6" t="s">
-        <v>892</v>
+        <v>896</v>
       </c>
       <c r="D112" s="6" t="s">
-        <v>893</v>
+        <v>897</v>
       </c>
       <c r="E112" s="6" t="s">
         <v>16</v>
@@ -9287,21 +9325,21 @@
         <v>317</v>
       </c>
       <c r="H112" s="6" t="s">
-        <v>894</v>
+        <v>898</v>
       </c>
     </row>
     <row r="113" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="7" t="s">
-        <v>895</v>
+        <v>899</v>
       </c>
       <c r="B113" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C113" s="6" t="s">
-        <v>896</v>
+        <v>900</v>
       </c>
       <c r="D113" s="6" t="s">
-        <v>897</v>
+        <v>901</v>
       </c>
       <c r="E113" s="6" t="s">
         <v>16</v>
@@ -9313,21 +9351,21 @@
         <v>317</v>
       </c>
       <c r="H113" s="6" t="s">
-        <v>898</v>
+        <v>902</v>
       </c>
     </row>
     <row r="114" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="7" t="s">
-        <v>899</v>
+        <v>903</v>
       </c>
       <c r="B114" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C114" s="6" t="s">
-        <v>900</v>
+        <v>904</v>
       </c>
       <c r="D114" s="6" t="s">
-        <v>901</v>
+        <v>905</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>16</v>
@@ -9339,21 +9377,21 @@
         <v>317</v>
       </c>
       <c r="H114" s="6" t="s">
-        <v>902</v>
+        <v>906</v>
       </c>
     </row>
     <row r="115" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="7" t="s">
-        <v>903</v>
+        <v>907</v>
       </c>
       <c r="B115" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C115" s="6" t="s">
-        <v>904</v>
+        <v>908</v>
       </c>
       <c r="D115" s="6" t="s">
-        <v>905</v>
+        <v>909</v>
       </c>
       <c r="E115" s="6" t="s">
         <v>16</v>
@@ -9365,21 +9403,21 @@
         <v>317</v>
       </c>
       <c r="H115" s="6" t="s">
-        <v>906</v>
+        <v>910</v>
       </c>
     </row>
     <row r="116" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="7" t="s">
-        <v>907</v>
+        <v>911</v>
       </c>
       <c r="B116" s="6" t="s">
         <v>27</v>
       </c>
       <c r="C116" s="6" t="s">
-        <v>908</v>
+        <v>912</v>
       </c>
       <c r="D116" s="6" t="s">
-        <v>909</v>
+        <v>913</v>
       </c>
       <c r="E116" s="6" t="s">
         <v>16</v>
@@ -9391,21 +9429,21 @@
         <v>317</v>
       </c>
       <c r="H116" s="6" t="s">
-        <v>910</v>
+        <v>914</v>
       </c>
     </row>
     <row r="117" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="7" t="s">
-        <v>911</v>
+        <v>915</v>
       </c>
       <c r="B117" s="6" t="s">
         <v>26</v>
       </c>
       <c r="C117" s="6" t="s">
-        <v>912</v>
+        <v>916</v>
       </c>
       <c r="D117" s="6" t="s">
-        <v>913</v>
+        <v>917</v>
       </c>
       <c r="E117" s="6" t="s">
         <v>16</v>
@@ -9417,21 +9455,21 @@
         <v>317</v>
       </c>
       <c r="H117" s="6" t="s">
-        <v>914</v>
+        <v>918</v>
       </c>
     </row>
     <row r="118" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="7" t="s">
-        <v>915</v>
+        <v>919</v>
       </c>
       <c r="B118" s="6" t="s">
         <v>28</v>
       </c>
       <c r="C118" s="6" t="s">
-        <v>916</v>
+        <v>920</v>
       </c>
       <c r="D118" s="6" t="s">
-        <v>917</v>
+        <v>921</v>
       </c>
       <c r="E118" s="6" t="s">
         <v>16</v>
@@ -9443,7 +9481,7 @@
         <v>317</v>
       </c>
       <c r="H118" s="6" t="s">
-        <v>918</v>
+        <v>922</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Give the filter row its own id
It was filed as FE-40, which was already the status-colour row, so
npm run register exited non-zero on a duplicate id — and the commit before
this one went in over that failure, which is the thing worth noting. The
same fault cost three commits of red verify on 18 Aug (SEC-04, SEC-05).

FE-41. The register is well-formed again and verify is green.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Things That Need Attention.xlsx
+++ b/docs/Things That Need Attention.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1905" uniqueCount="956">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1913" uniqueCount="960">
   <si>
     <t>AussieMed — things that need attention</t>
   </si>
@@ -2475,6 +2475,18 @@
   </si>
   <si>
     <t>Built 17 Aug 2026 at the client's request: a country dropdown, the states of each country, and the dialling prefix, on every form that asks for an address. One shared component across the branch form, the supplier form and checkout, because four forms reading these for themselves is how four ideas of an address arise. All 152 countries are listed, with the UAE pinned first — nearly every address here is Emirati and a form whose commonest answer is 230 rows down gets the wrong answer. Subdivisions are held only for the GCC and the countries goods come from, sixteen in all: the full ISO 3166-2 set is several thousand entries and would be shipped into every form that renders a picker, which is the mistake BE-47 was about. A country with no list gets a free-text box labelled with the word that country uses, so it degrades honestly. The label follows the country — Emirate for the UAE, Governorate for Oman, State for India, Province for China — and changing the country clears the subdivision, because Dubai left sitting under Germany looks answered and is not. The dialling prefix is shown beside the phone rather than inside it, and the domestic leading zero is dropped when the two are joined: +971 050... is not a number anyone can ring and is exactly what concatenating the halves gives. Existing free-text values are matched case-insensitively and kept as typed when unrecognised, so nothing already delivering parcels is lost. Rules are pure and tested in geo.ts, 37 tests. Verified by placing a real order to Muscat and reading the stored snapshot and the printed delivery note.</t>
+  </si>
+  <si>
+    <t>FE-41</t>
+  </si>
+  <si>
+    <t>The filter bar is a box of its own, opened where the buyer clicked</t>
+  </si>
+  <si>
+    <t>The filter was an unframed column that scrolled with the page. At 445 categories, arriving from a front-page tile landed a buyer at the top of an alphabetical list with the category they had just chosen somewhere below the fold, and scrolling to find it scrolled the products away as well.</t>
+  </si>
+  <si>
+    <t>Built 19 Aug 2026 at the client's request. Three things, and the third is the one that matters. It is BOXED: a bordered panel with its own header carrying a Clear all that resets category, brand and availability together, replacing the clear-category link buried in the list. It SCROLLS ON ITS OWN: sticky beside the results, capped at the height of the screen, so a fifty-row department can be read without the products leaving with it. And it OPENS ON WHAT WAS CHOSEN: the active entry is marked at all three levels and src/components/FilterScroll.tsx scrolls the box — not the page — to it on mount, a third of the way down so the shelves beneath an open category are visible too, and not at all when it is already in view. Deliberately scrollTop rather than scrollIntoView, which scrolls every ancestor that can scroll and drags a sticky sidebar's whole page down with it. CONSISTENCY IS STRUCTURAL rather than a convention: the frame moved out of the products page and into the component, so the one route it appears on — every category, every search, every brand view — cannot dress it differently on one of them. Verified by arriving the way a buyer does, clicking Dental on the front page and finding it in view, and by a deep link to a third-level shelf, which opens the box scrolled to Hand Files with the page still at the top.</t>
   </si>
   <si>
     <t>FN-08</t>
@@ -3391,7 +3403,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="3">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3415,7 +3427,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="3">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -6529,7 +6541,7 @@
   <sheetPr>
     <tabColor rgb="FF146C43"/>
   </sheetPr>
-  <dimension ref="A1:H125"/>
+  <dimension ref="A1:H126"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -8912,7 +8924,7 @@
         <v>820</v>
       </c>
       <c r="B92" s="6" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C92" s="6" t="s">
         <v>821</v>
@@ -9198,7 +9210,7 @@
         <v>864</v>
       </c>
       <c r="B103" s="6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C103" s="6" t="s">
         <v>865</v>
@@ -9302,7 +9314,7 @@
         <v>880</v>
       </c>
       <c r="B107" s="6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C107" s="6" t="s">
         <v>881</v>
@@ -9313,8 +9325,8 @@
       <c r="E107" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F107" s="10" t="s">
-        <v>241</v>
+      <c r="F107" s="9" t="s">
+        <v>98</v>
       </c>
       <c r="G107" s="11" t="s">
         <v>310</v>
@@ -9458,7 +9470,7 @@
         <v>904</v>
       </c>
       <c r="B113" s="6" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C113" s="6" t="s">
         <v>905</v>
@@ -9466,8 +9478,8 @@
       <c r="D113" s="6" t="s">
         <v>906</v>
       </c>
-      <c r="E113" s="7" t="s">
-        <v>13</v>
+      <c r="E113" s="6" t="s">
+        <v>16</v>
       </c>
       <c r="F113" s="10" t="s">
         <v>241</v>
@@ -9518,8 +9530,8 @@
       <c r="D115" s="6" t="s">
         <v>914</v>
       </c>
-      <c r="E115" s="6" t="s">
-        <v>16</v>
+      <c r="E115" s="7" t="s">
+        <v>13</v>
       </c>
       <c r="F115" s="10" t="s">
         <v>241</v>
@@ -9718,7 +9730,7 @@
         <v>944</v>
       </c>
       <c r="B123" s="6" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="C123" s="6" t="s">
         <v>945</v>
@@ -9744,7 +9756,7 @@
         <v>948</v>
       </c>
       <c r="B124" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C124" s="6" t="s">
         <v>949</v>
@@ -9770,7 +9782,7 @@
         <v>952</v>
       </c>
       <c r="B125" s="6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C125" s="6" t="s">
         <v>953</v>
@@ -9791,8 +9803,34 @@
         <v>955</v>
       </c>
     </row>
+    <row r="126" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A126" s="7" t="s">
+        <v>956</v>
+      </c>
+      <c r="B126" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C126" s="6" t="s">
+        <v>957</v>
+      </c>
+      <c r="D126" s="6" t="s">
+        <v>958</v>
+      </c>
+      <c r="E126" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F126" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="G126" s="11" t="s">
+        <v>310</v>
+      </c>
+      <c r="H126" s="6" t="s">
+        <v>959</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H125"/>
+  <autoFilter ref="A1:H126"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>